<commit_message>
Rebuild D4's composite contribution via state-name join
Swaps D4's source from the superseded CPM-only dimension4_final.csv to
the current pd_revised methodology, joined by state name like D2/D3/D5
were in the prior composite rebuild. 8 states change composite tier;
Dashboard summary stats updated to match. Dossier text was already
accurate and needed no change, it already described pd_revised.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/composite/PSAI_CompositeScores_Rebuilt.xlsx
+++ b/composite/PSAI_CompositeScores_Rebuilt.xlsx
@@ -478,7 +478,7 @@
         <v>38.5</v>
       </c>
       <c r="E2" t="n">
-        <v>91.5</v>
+        <v>78.5</v>
       </c>
       <c r="F2" t="n">
         <v>70</v>
@@ -509,7 +509,7 @@
         <v>13.6</v>
       </c>
       <c r="E3" t="n">
-        <v>38.5</v>
+        <v>77</v>
       </c>
       <c r="F3" t="n">
         <v>87.5</v>
@@ -520,7 +520,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>New Jersey</t>
+          <t>California</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
         <v>22.7</v>
       </c>
       <c r="E4" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
@@ -571,7 +571,7 @@
         <v>61.5</v>
       </c>
       <c r="E5" t="n">
-        <v>91.5</v>
+        <v>75</v>
       </c>
       <c r="F5" t="n">
         <v>55</v>
@@ -582,7 +582,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>New Jersey</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
         <v>30</v>
       </c>
       <c r="E6" t="n">
-        <v>50</v>
+        <v>96</v>
       </c>
       <c r="F6" t="n">
         <v>85</v>
@@ -633,7 +633,7 @@
         <v>35</v>
       </c>
       <c r="E7" t="n">
-        <v>94</v>
+        <v>54</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
@@ -644,7 +644,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Pennsylvania</t>
+          <t>Wisconsin</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
         <v>52.1</v>
       </c>
       <c r="E8" t="n">
-        <v>46</v>
+        <v>84.5</v>
       </c>
       <c r="F8" t="n">
         <v>60</v>
@@ -675,7 +675,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Maryland</t>
+          <t>Minnesota</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -725,7 +725,7 @@
         <v>38.5</v>
       </c>
       <c r="E9" t="n">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="F9" t="n">
         <v>100</v>
@@ -736,7 +736,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>Pennsylvania</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -782,7 +782,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Iowa</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
         <v>50</v>
       </c>
       <c r="E11" t="n">
-        <v>66.5</v>
+        <v>45</v>
       </c>
       <c r="F11" t="n">
         <v>40</v>
@@ -813,7 +813,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Maryland</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
         <v>28.6</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="F12" t="n">
         <v>70</v>
@@ -844,7 +844,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>North Dakota</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         <v>43.3</v>
       </c>
       <c r="E13" t="n">
-        <v>46</v>
+        <v>49.5</v>
       </c>
       <c r="F13" t="n">
         <v>100</v>
@@ -875,7 +875,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>North Carolina</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
         <v>31.8</v>
       </c>
       <c r="E14" t="n">
-        <v>66.5</v>
+        <v>72.5</v>
       </c>
       <c r="F14" t="n">
         <v>23.5</v>
@@ -906,7 +906,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>New Mexico</t>
+          <t>Massachusetts</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
         <v>45.5</v>
       </c>
       <c r="E15" t="n">
-        <v>94</v>
+        <v>88.5</v>
       </c>
       <c r="F15" t="n">
         <v>64.7</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>Alabama</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
         <v>42.9</v>
       </c>
       <c r="E16" t="n">
-        <v>96</v>
+        <v>90.5</v>
       </c>
       <c r="F16" t="n">
         <v>81.2</v>
@@ -968,7 +968,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Wyoming</t>
+          <t>New Mexico</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
         <v>27.3</v>
       </c>
       <c r="E17" t="n">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F17" t="n">
         <v>20</v>
@@ -999,7 +999,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Massachusetts</t>
+          <t>Montana</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
         <v>32.1</v>
       </c>
       <c r="E18" t="n">
-        <v>91.5</v>
+        <v>78.5</v>
       </c>
       <c r="F18" t="n">
         <v>100</v>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>North Dakota</t>
+          <t>Idaho</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
         <v>33.3</v>
       </c>
       <c r="E19" t="n">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="F19" t="n">
         <v>85</v>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Idaho</t>
+          <t>Michigan</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
         <v>33.1</v>
       </c>
       <c r="E20" t="n">
-        <v>69</v>
+        <v>82.5</v>
       </c>
       <c r="F20" t="n">
         <v>41.2</v>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Colorado</t>
+          <t>Wyoming</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1112,7 @@
         <v>31.5</v>
       </c>
       <c r="E21" t="n">
-        <v>46</v>
+        <v>77</v>
       </c>
       <c r="F21" t="n">
         <v>55</v>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Vermont</t>
+          <t>New York</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
         <v>42.6</v>
       </c>
       <c r="E22" t="n">
-        <v>69</v>
+        <v>47.5</v>
       </c>
       <c r="F22" t="n">
         <v>33.3</v>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>New Hampshire</t>
+          <t>Tennessee</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
         <v>32</v>
       </c>
       <c r="E23" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F23" t="n">
         <v>57.1</v>
@@ -1205,7 +1205,7 @@
         <v>30</v>
       </c>
       <c r="E24" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Montana</t>
+          <t>Delaware</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
         <v>25</v>
       </c>
       <c r="E25" t="n">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>Alaska</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
         <v>23.1</v>
       </c>
       <c r="E27" t="n">
-        <v>96</v>
+        <v>90.5</v>
       </c>
       <c r="F27" t="n">
         <v>85</v>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>South Dakota</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
         <v>35.7</v>
       </c>
       <c r="E28" t="n">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="F28" t="n">
         <v>85</v>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Kentucky</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
         <v>22.2</v>
       </c>
       <c r="E29" t="n">
-        <v>66.5</v>
+        <v>72.5</v>
       </c>
       <c r="F29" t="n">
         <v>65</v>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Connecticut</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
         <v>53.9</v>
       </c>
       <c r="E30" t="n">
-        <v>94</v>
+        <v>88.5</v>
       </c>
       <c r="F30" t="n">
         <v>87.5</v>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Mississippi</t>
+          <t>Vermont</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
         <v>45</v>
       </c>
       <c r="E31" t="n">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="F31" t="n">
         <v>40</v>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Hawaii</t>
+          <t>New Hampshire</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
         <v>51.5</v>
       </c>
       <c r="E32" t="n">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F32" t="n">
         <v>100</v>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Hawaii</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
         <v>46.2</v>
       </c>
       <c r="E33" t="n">
-        <v>86.5</v>
+        <v>73.5</v>
       </c>
       <c r="F33" t="n">
         <v>35</v>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Alaska</t>
+          <t>Mississippi</t>
         </is>
       </c>
     </row>
@@ -1515,7 +1515,7 @@
         <v>28.6</v>
       </c>
       <c r="E34" t="n">
-        <v>41.5</v>
+        <v>80</v>
       </c>
       <c r="F34" t="n">
         <v>70</v>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>South Dakota</t>
+          <t>Maine</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Indiana</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1577,7 @@
         <v>43.8</v>
       </c>
       <c r="E36" t="n">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="F36" t="n">
         <v>66.7</v>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Colorado</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
         <v>30.6</v>
       </c>
       <c r="E37" t="n">
-        <v>75</v>
+        <v>53.5</v>
       </c>
       <c r="F37" t="n">
         <v>43.8</v>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Delaware</t>
+          <t>Kansas</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
         <v>12.5</v>
       </c>
       <c r="E38" t="n">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="F38" t="n">
         <v>50</v>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Arkansas</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
         <v>33.3</v>
       </c>
       <c r="E39" t="n">
-        <v>69</v>
+        <v>82.5</v>
       </c>
       <c r="F39" t="n">
         <v>85</v>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Rhode Island</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Connecticut</t>
+          <t>Nebraska</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
         <v>42.5</v>
       </c>
       <c r="E41" t="n">
-        <v>44</v>
+        <v>82.5</v>
       </c>
       <c r="F41" t="n">
         <v>20</v>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Maine</t>
+          <t>Georgia</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
         <v>48.7</v>
       </c>
       <c r="E42" t="n">
-        <v>96</v>
+        <v>90.5</v>
       </c>
       <c r="F42" t="n">
         <v>50</v>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Arizona</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
         <v>64.40000000000001</v>
       </c>
       <c r="E43" t="n">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="F43" t="n">
         <v>100</v>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Louisiana</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1825,7 @@
         <v>37.5</v>
       </c>
       <c r="E44" t="n">
-        <v>71</v>
+        <v>88.5</v>
       </c>
       <c r="F44" t="n">
         <v>88.2</v>
@@ -1856,7 +1856,7 @@
         <v>29.8</v>
       </c>
       <c r="E45" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F45" t="n">
         <v>46.2</v>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>South Carolina</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
         <v>33.3</v>
       </c>
       <c r="E46" t="n">
-        <v>75</v>
+        <v>53.5</v>
       </c>
       <c r="F46" t="n">
         <v>85</v>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>South Carolina</t>
+          <t>Florida</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
         <v>15.4</v>
       </c>
       <c r="E47" t="n">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Louisiana</t>
+          <t>Missouri</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
         <v>29.2</v>
       </c>
       <c r="E48" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F48" t="n">
         <v>70</v>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>Utah</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
         <v>13.6</v>
       </c>
       <c r="E49" t="n">
-        <v>71</v>
+        <v>84.5</v>
       </c>
       <c r="F49" t="n">
         <v>100</v>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Rhode Island</t>
+          <t>Texas</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
         <v>30.8</v>
       </c>
       <c r="E50" t="n">
-        <v>69</v>
+        <v>71.5</v>
       </c>
       <c r="F50" t="n">
         <v>10</v>
@@ -2022,7 +2022,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Ohio</t>
+          <t>District of Columbia</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
         <v>34.6</v>
       </c>
       <c r="E51" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F51" t="n">
         <v>100</v>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>District of Columbia</t>
+          <t>Ohio</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
         <v>44</v>
       </c>
       <c r="E52" t="n">
-        <v>91.5</v>
+        <v>75</v>
       </c>
       <c r="F52" t="n">
         <v>30.8</v>

</xml_diff>

<commit_message>
Fix D.C. D4 zero, regenerate all composite outputs, polish for review
- D.C. D4 now scored on the PD half alone (70) instead of 0, per D4's
  never-default-D.C.-to-zero rule; composite 40.3 -> 50.8, rank 49 -> 35
- Regenerate workbook (with cached values), scores CSV, dashboard data,
  alternatives and robustness results from one run (composite/regenerate.py)
- Unify District of Columbia spelling across data files
- Move Methods Spec up; add answer options to Questions 02-06
- Add spot_check_protocol.md and CHANGELOG.md

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/composite/PSAI_CompositeScores_Rebuilt.xlsx
+++ b/composite/PSAI_CompositeScores_Rebuilt.xlsx
@@ -485,7 +485,7 @@
       </c>
       <c r="G2">
         <f>SUMPRODUCT(B2:F2, $L$9:$P$9)</f>
-        <v/>
+        <v>60.08954521908776</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -516,7 +516,7 @@
       </c>
       <c r="G3">
         <f>SUMPRODUCT(B3:F3, $L$9:$P$9)</f>
-        <v/>
+        <v>55.445</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -547,7 +547,7 @@
       </c>
       <c r="G4">
         <f>SUMPRODUCT(B4:F4, $L$9:$P$9)</f>
-        <v/>
+        <v>47.05583149332072</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="G5">
         <f>SUMPRODUCT(B5:F5, $L$9:$P$9)</f>
-        <v/>
+        <v>48.73571428571428</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
       </c>
       <c r="G6">
         <f>SUMPRODUCT(B6:F6, $L$9:$P$9)</f>
-        <v/>
+        <v>70.65782778129726</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -640,7 +640,7 @@
       </c>
       <c r="G7">
         <f>SUMPRODUCT(B7:F7, $L$9:$P$9)</f>
-        <v/>
+        <v>50.71384132595445</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -671,7 +671,7 @@
       </c>
       <c r="G8">
         <f>SUMPRODUCT(B8:F8, $L$9:$P$9)</f>
-        <v/>
+        <v>53.08324253663906</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -732,7 +732,7 @@
       </c>
       <c r="G9">
         <f>SUMPRODUCT(B9:F9, $L$9:$P$9)</f>
-        <v/>
+        <v>55.861358049238376</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -771,14 +771,14 @@
         <v>29.2</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>70.0</v>
       </c>
       <c r="F10" t="n">
         <v>22.2</v>
       </c>
       <c r="G10">
         <f>SUMPRODUCT(B10:F10, $L$9:$P$9)</f>
-        <v/>
+        <v>50.806836759652995</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -809,7 +809,7 @@
       </c>
       <c r="G11">
         <f>SUMPRODUCT(B11:F11, $L$9:$P$9)</f>
-        <v/>
+        <v>43.130141566073085</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -840,7 +840,7 @@
       </c>
       <c r="G12">
         <f>SUMPRODUCT(B12:F12, $L$9:$P$9)</f>
-        <v/>
+        <v>47.29344326898824</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
       </c>
       <c r="G13">
         <f>SUMPRODUCT(B13:F13, $L$9:$P$9)</f>
-        <v/>
+        <v>52.03348868593249</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -902,7 +902,7 @@
       </c>
       <c r="G14">
         <f>SUMPRODUCT(B14:F14, $L$9:$P$9)</f>
-        <v/>
+        <v>59.038000000000004</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -933,7 +933,7 @@
       </c>
       <c r="G15">
         <f>SUMPRODUCT(B15:F15, $L$9:$P$9)</f>
-        <v/>
+        <v>71.10407763628673</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
       </c>
       <c r="G16">
         <f>SUMPRODUCT(B16:F16, $L$9:$P$9)</f>
-        <v/>
+        <v>51.165</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -995,7 +995,7 @@
       </c>
       <c r="G17">
         <f>SUMPRODUCT(B17:F17, $L$9:$P$9)</f>
-        <v/>
+        <v>64.28</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="G18">
         <f>SUMPRODUCT(B18:F18, $L$9:$P$9)</f>
-        <v/>
+        <v>50.013000000000005</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="G19">
         <f>SUMPRODUCT(B19:F19, $L$9:$P$9)</f>
-        <v/>
+        <v>53.242</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="G20">
         <f>SUMPRODUCT(B20:F20, $L$9:$P$9)</f>
-        <v/>
+        <v>46.3235945748366</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="G21">
         <f>SUMPRODUCT(B21:F21, $L$9:$P$9)</f>
-        <v/>
+        <v>51.312522091545134</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="G22">
         <f>SUMPRODUCT(B22:F22, $L$9:$P$9)</f>
-        <v/>
+        <v>63.18349899783583</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="G23">
         <f>SUMPRODUCT(B23:F23, $L$9:$P$9)</f>
-        <v/>
+        <v>60.09856114840955</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="G24">
         <f>SUMPRODUCT(B24:F24, $L$9:$P$9)</f>
-        <v/>
+        <v>58.296</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="G25">
         <f>SUMPRODUCT(B25:F25, $L$9:$P$9)</f>
-        <v/>
+        <v>67.6</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="G26">
         <f>SUMPRODUCT(B26:F26, $L$9:$P$9)</f>
-        <v/>
+        <v>51.8114610388326</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="G27">
         <f>SUMPRODUCT(B27:F27, $L$9:$P$9)</f>
-        <v/>
+        <v>41.903</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="G28">
         <f>SUMPRODUCT(B28:F28, $L$9:$P$9)</f>
-        <v/>
+        <v>59.230000000000004</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="G29">
         <f>SUMPRODUCT(B29:F29, $L$9:$P$9)</f>
-        <v/>
+        <v>47.429</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="G30">
         <f>SUMPRODUCT(B30:F30, $L$9:$P$9)</f>
-        <v/>
+        <v>69.588</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G31">
         <f>SUMPRODUCT(B31:F31, $L$9:$P$9)</f>
-        <v/>
+        <v>52.8240486427539</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="G32">
         <f>SUMPRODUCT(B32:F32, $L$9:$P$9)</f>
-        <v/>
+        <v>68.6299091124736</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="G33">
         <f>SUMPRODUCT(B33:F33, $L$9:$P$9)</f>
-        <v/>
+        <v>59.307</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="G34">
         <f>SUMPRODUCT(B34:F34, $L$9:$P$9)</f>
-        <v/>
+        <v>57.74878015264153</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="G35">
         <f>SUMPRODUCT(B35:F35, $L$9:$P$9)</f>
-        <v/>
+        <v>61.15267215441075</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -1584,11 +1584,11 @@
       </c>
       <c r="G36">
         <f>SUMPRODUCT(B36:F36, $L$9:$P$9)</f>
-        <v/>
+        <v>63.173</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Colorado</t>
+          <t>District of Columbia</t>
         </is>
       </c>
     </row>
@@ -1615,11 +1615,11 @@
       </c>
       <c r="G37">
         <f>SUMPRODUCT(B37:F37, $L$9:$P$9)</f>
-        <v/>
+        <v>39.351</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Colorado</t>
         </is>
       </c>
     </row>
@@ -1646,11 +1646,11 @@
       </c>
       <c r="G38">
         <f>SUMPRODUCT(B38:F38, $L$9:$P$9)</f>
-        <v/>
+        <v>43.764</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Kansas</t>
         </is>
       </c>
     </row>
@@ -1677,11 +1677,11 @@
       </c>
       <c r="G39">
         <f>SUMPRODUCT(B39:F39, $L$9:$P$9)</f>
-        <v/>
+        <v>68.51636744984543</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Rhode Island</t>
+          <t>Arkansas</t>
         </is>
       </c>
     </row>
@@ -1708,11 +1708,11 @@
       </c>
       <c r="G40">
         <f>SUMPRODUCT(B40:F40, $L$9:$P$9)</f>
-        <v/>
+        <v>66.42871944368238</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Rhode Island</t>
         </is>
       </c>
     </row>
@@ -1739,11 +1739,11 @@
       </c>
       <c r="G41">
         <f>SUMPRODUCT(B41:F41, $L$9:$P$9)</f>
-        <v/>
+        <v>48.45480510797095</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Nebraska</t>
         </is>
       </c>
     </row>
@@ -1770,11 +1770,11 @@
       </c>
       <c r="G42">
         <f>SUMPRODUCT(B42:F42, $L$9:$P$9)</f>
-        <v/>
+        <v>43.530438626141716</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Georgia</t>
         </is>
       </c>
     </row>
@@ -1801,11 +1801,11 @@
       </c>
       <c r="G43">
         <f>SUMPRODUCT(B43:F43, $L$9:$P$9)</f>
-        <v/>
+        <v>54.118</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Louisiana</t>
+          <t>Arizona</t>
         </is>
       </c>
     </row>
@@ -1832,11 +1832,11 @@
       </c>
       <c r="G44">
         <f>SUMPRODUCT(B44:F44, $L$9:$P$9)</f>
-        <v/>
+        <v>57.18164608660909</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Oklahoma</t>
+          <t>Louisiana</t>
         </is>
       </c>
     </row>
@@ -1863,11 +1863,11 @@
       </c>
       <c r="G45">
         <f>SUMPRODUCT(B45:F45, $L$9:$P$9)</f>
-        <v/>
+        <v>41.50396200867281</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>South Carolina</t>
+          <t>Oklahoma</t>
         </is>
       </c>
     </row>
@@ -1894,11 +1894,11 @@
       </c>
       <c r="G46">
         <f>SUMPRODUCT(B46:F46, $L$9:$P$9)</f>
-        <v/>
+        <v>41.71547444517231</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>South Carolina</t>
         </is>
       </c>
     </row>
@@ -1925,11 +1925,11 @@
       </c>
       <c r="G47">
         <f>SUMPRODUCT(B47:F47, $L$9:$P$9)</f>
-        <v/>
+        <v>52.93084517302114</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>Florida</t>
         </is>
       </c>
     </row>
@@ -1956,11 +1956,11 @@
       </c>
       <c r="G48">
         <f>SUMPRODUCT(B48:F48, $L$9:$P$9)</f>
-        <v/>
+        <v>55.167713334323366</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Missouri</t>
         </is>
       </c>
     </row>
@@ -1987,11 +1987,11 @@
       </c>
       <c r="G49">
         <f>SUMPRODUCT(B49:F49, $L$9:$P$9)</f>
-        <v/>
+        <v>56.66479341896031</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Utah</t>
         </is>
       </c>
     </row>
@@ -2018,11 +2018,11 @@
       </c>
       <c r="G50">
         <f>SUMPRODUCT(B50:F50, $L$9:$P$9)</f>
-        <v/>
+        <v>32.713</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>District of Columbia</t>
+          <t>Texas</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="G51">
         <f>SUMPRODUCT(B51:F51, $L$9:$P$9)</f>
-        <v/>
+        <v>68.426</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="G52">
         <f>SUMPRODUCT(B52:F52, $L$9:$P$9)</f>
-        <v/>
+        <v>58.242</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>

</xml_diff>